<commit_message>
Condo Assistant: update model with real client distribution + $500 enterprise flat rate (~$4.1M ARR)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_files/Condo_Assistant_SaaS_Model.xlsx
+++ b/project_files/Condo_Assistant_SaaS_Model.xlsx
@@ -15,9 +15,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="87">
-  <si>
-    <t>CONDO ASSISTANT — PRICING (per unit / month)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="90">
+  <si>
+    <t>CONDO ASSISTANT — PRICING</t>
   </si>
   <si>
     <t>Band</t>
@@ -62,19 +62,25 @@
     <t>20–49 units</t>
   </si>
   <si>
-    <t>Tier 4</t>
-  </si>
-  <si>
-    <t>50+ units</t>
-  </si>
-  <si>
-    <t>Note: single product = Condo Assistant OR Auto Email ($15 base). Bundle = both ($25 base). Volume breaks at 3, 10, 20, 50 units.</t>
-  </si>
-  <si>
-    <t>REVENUE MODEL — at full penetration of target clients</t>
-  </si>
-  <si>
-    <t>Total Target Clients</t>
+    <t>Enterprise</t>
+  </si>
+  <si>
+    <t>50–100 units</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>FLAT $500/mo</t>
+  </si>
+  <si>
+    <t>Enterprise = clients with 50–100 units pay a flat $500/mo (≈$6.67/unit at 75 units). 100+ units = custom.</t>
+  </si>
+  <si>
+    <t>Single product = Condo Assistant OR Auto Email. Bundle = both. Bigger discount kicks in at 20+ units.</t>
+  </si>
+  <si>
+    <t>REVENUE MODEL — at full penetration</t>
   </si>
   <si>
     <t>Bundle Adoption %</t>
@@ -83,31 +89,34 @@
     <t>Single-Product %</t>
   </si>
   <si>
-    <t>% Clients</t>
+    <t>Enterprise Flat Rate ($/mo)</t>
   </si>
   <si>
     <t># Clients</t>
   </si>
   <si>
-    <t>Avg Units/Client</t>
+    <t>Avg Units</t>
   </si>
   <si>
     <t>Total Units</t>
   </si>
   <si>
-    <t>Bundle $/unit</t>
-  </si>
-  <si>
-    <t>Single $/unit</t>
-  </si>
-  <si>
-    <t>Blended $/unit</t>
-  </si>
-  <si>
-    <t>Monthly Revenue</t>
-  </si>
-  <si>
-    <t>Annual Revenue</t>
+    <t>Bundle $/u</t>
+  </si>
+  <si>
+    <t>Single $/u</t>
+  </si>
+  <si>
+    <t>Blended $/u</t>
+  </si>
+  <si>
+    <t>Monthly Rev</t>
+  </si>
+  <si>
+    <t>Annual Rev</t>
+  </si>
+  <si>
+    <t>flat</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -128,7 +137,7 @@
     <t>COGS / Unit / Month (AI + hosting + email)</t>
   </si>
   <si>
-    <t>Stripe Fee (% of revenue, blended)</t>
+    <t>Stripe Fee (% of revenue)</t>
   </si>
   <si>
     <t>Gross Profit / Unit / Month</t>
@@ -152,7 +161,7 @@
     <t>CAC / LTV</t>
   </si>
   <si>
-    <t>CAC — Customer Acquisition Cost</t>
+    <t>CAC</t>
   </si>
   <si>
     <t>Monthly Churn %</t>
@@ -164,13 +173,13 @@
     <t>LTV (gross profit)</t>
   </si>
   <si>
-    <t>LTV : CAC Ratio</t>
+    <t>LTV : CAC</t>
   </si>
   <si>
     <t>CAC Payback (months)</t>
   </si>
   <si>
-    <t>ROLLOUT RAMP TO 5,000 CLIENTS</t>
+    <t>ROLLOUT RAMP</t>
   </si>
   <si>
     <t>Year</t>
@@ -179,7 +188,7 @@
     <t>Clients</t>
   </si>
   <si>
-    <t>% of Target</t>
+    <t>% Target</t>
   </si>
   <si>
     <t>Est. ARR</t>
@@ -191,61 +200,58 @@
     <t>Year 1</t>
   </si>
   <si>
-    <t>Pilot &amp; early adopters — WPM referrals, CO STR Facebook groups, VRBO/Airbnb host DMs</t>
+    <t>Pilot &amp; early adopters — WPM referrals, CO STR groups, host DMs (near-zero CAC)</t>
   </si>
   <si>
     <t>Year 2</t>
   </si>
   <si>
-    <t>Scale — Google Business + SEO, cold outreach to PM cos, Escapia/Guesty affiliate program</t>
+    <t>Scale — PM/software partners + Escapia/Guesty affiliates (Option C)</t>
   </si>
   <si>
     <t>Year 3</t>
   </si>
   <si>
-    <t>Full penetration — paid search, demo videos, Product Hunt, referral flywheel</t>
-  </si>
-  <si>
-    <t>HOW TO USE</t>
-  </si>
-  <si>
-    <t>Editable inputs</t>
-  </si>
-  <si>
-    <t>Pricing tiers, client distribution %, avg units/client, bundle adoption %, COGS, Stripe %, CAC, churn, ramp targets. Everything else calculates.</t>
+    <t>Full penetration — paid acquisition + referral flywheel (Option B)</t>
   </si>
   <si>
     <t>PRICING</t>
   </si>
   <si>
-    <t>$15 Condo Assistant · $15 Auto Email · $25 both (bundle)</t>
-  </si>
-  <si>
-    <t>Volume breaks</t>
-  </si>
-  <si>
-    <t>3, 10, 20, 50 units — per-unit price drops ~12% / 20% / 30% / 40% off bundle base</t>
-  </si>
-  <si>
-    <t>REVENUE MODEL</t>
-  </si>
-  <si>
-    <t>Target clients</t>
-  </si>
-  <si>
-    <t>5,000 VRBO clients (owners + small PM companies)</t>
-  </si>
-  <si>
-    <t>Client distribution</t>
-  </si>
-  <si>
-    <t>Illustrative: 70% have 1–2 units, 20% have 3–9, 6% have 10–19, 3% have 20–49, 1% have 50+ — replace with real market data</t>
-  </si>
-  <si>
-    <t>Bundle adoption</t>
-  </si>
-  <si>
-    <t>65% take the bundle, 35% take a single product (editable)</t>
+    <t>Per-unit bands</t>
+  </si>
+  <si>
+    <t>1–2 $25 · 3–9 $22 · 10–19 $20 · 20–49 $14 (bundle). Single product ~$6 less. Bigger discount at 20+.</t>
+  </si>
+  <si>
+    <t>Enterprise (50–100 units)</t>
+  </si>
+  <si>
+    <t>FLAT $500/mo per client (≈$6.67/unit at 75 units). 100+ units = custom quote.</t>
+  </si>
+  <si>
+    <t>CLIENT DISTRIBUTION (your numbers)</t>
+  </si>
+  <si>
+    <t>4,000 clients</t>
+  </si>
+  <si>
+    <t>500 clients</t>
+  </si>
+  <si>
+    <t>300 clients</t>
+  </si>
+  <si>
+    <t>200 clients</t>
+  </si>
+  <si>
+    <t>50 clients (seeded — the "rest"; adjust as needed)</t>
+  </si>
+  <si>
+    <t>Avg units/client</t>
+  </si>
+  <si>
+    <t>Illustrative per band (1.5 / 5 / 13 / 30 / 75) — refine with real data</t>
   </si>
   <si>
     <t>UNIT ECONOMICS</t>
@@ -254,28 +260,31 @@
     <t>COGS/unit/mo</t>
   </si>
   <si>
-    <t>$3 placeholder — Claude API + hosting (Vercel/Supabase) + Resend email, per unit</t>
+    <t>$3 placeholder — Claude API + hosting + Resend email</t>
   </si>
   <si>
     <t>Stripe</t>
   </si>
   <si>
-    <t>~3.5% blended (2.9% + $0.30/txn). You researched net-per-plan earlier.</t>
+    <t>~3.5% blended (2.9% + $0.30/txn)</t>
   </si>
   <si>
     <t>CAC / churn</t>
   </si>
   <si>
-    <t>$150 CAC, 3% monthly churn — illustrative SaaS defaults; refine with real funnel data</t>
-  </si>
-  <si>
-    <t>IMPORTANT</t>
-  </si>
-  <si>
-    <t>All numbers are illustrative</t>
-  </si>
-  <si>
-    <t>This is a planning model to show Alex the shape of the business. Distribution, COGS, CAC and churn are estimates — replace with real data as it comes in.</t>
+    <t>$150 CAC, 3% monthly churn — illustrative</t>
+  </si>
+  <si>
+    <t>NOTE — pricing cliff</t>
+  </si>
+  <si>
+    <t>A 49-unit client (per-unit) can pay more than a 50-unit client (flat $500). Intentional "graduate to enterprise" discount, but watch the boundary.</t>
+  </si>
+  <si>
+    <t>All numbers illustrative</t>
+  </si>
+  <si>
+    <t>Planning model to show Alex. Replace estimates with real data as it comes in.</t>
   </si>
 </sst>
 </file>
@@ -350,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -373,7 +382,6 @@
     <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -735,13 +743,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="4" width="20" style="1" customWidth="1"/>
-    <col min="5" max="5" width="22" style="1" customWidth="1"/>
+    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="18" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="2" customWidth="1"/>
   </cols>
   <sheetData>
@@ -842,13 +850,13 @@
         <v>14</v>
       </c>
       <c r="C7" s="1">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="D7" s="1">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="E7" s="1">
-        <v>17.5</v>
+        <v>14</v>
       </c>
       <c r="F7" s="2">
         <f>1-E7/$E$4</f>
@@ -861,22 +869,27 @@
       <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="1">
-        <v>9</v>
-      </c>
-      <c r="D8" s="1">
-        <v>9</v>
-      </c>
-      <c r="E8" s="1">
-        <v>15</v>
+      <c r="C8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="F8" s="2">
-        <f>1-E8/$E$4</f>
+        <f>1-(500/75)/E4</f>
       </c>
     </row>
     <row r="10" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>17</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -887,334 +900,307 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="12" style="2" customWidth="1"/>
-    <col min="3" max="3" width="12" style="11" customWidth="1"/>
-    <col min="4" max="4" width="14" style="12" customWidth="1"/>
-    <col min="5" max="5" width="12" style="11" customWidth="1"/>
-    <col min="6" max="8" width="14" style="1" customWidth="1"/>
-    <col min="9" max="10" width="16" style="13" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" style="11" customWidth="1"/>
+    <col min="3" max="3" width="14" style="12" customWidth="1"/>
+    <col min="4" max="4" width="12" style="11" customWidth="1"/>
+    <col min="5" max="5" width="14" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14" style="1" customWidth="1"/>
+    <col min="8" max="9" width="16" style="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="14"/>
+        <v>21</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="H1" s="16"/>
       <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="2">
-        <v>5000</v>
-      </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="11"/>
+        <v>22</v>
+      </c>
+      <c r="B3" s="11">
+        <v>0.65</v>
+      </c>
+      <c r="C3" s="12"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="H3" s="13"/>
       <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="2">
-        <v>0.65</v>
-      </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="B4" s="11">
+        <f>1-B3</f>
+      </c>
+      <c r="C4" s="12"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="H4" s="13"/>
       <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="2">
-        <f>1-B4</f>
-      </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="11"/>
+        <v>24</v>
+      </c>
+      <c r="B5" s="11">
+        <v>500</v>
+      </c>
+      <c r="C5" s="12"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
+      <c r="H5" s="13"/>
       <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-    </row>
-    <row r="7" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="18" t="s">
+      <c r="B7" s="18" t="s">
         <v>25</v>
       </c>
+      <c r="C7" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>28</v>
+      </c>
       <c r="F7" s="8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>31</v>
       </c>
       <c r="I7" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J7" s="20" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="2">
-        <v>0.7</v>
-      </c>
-      <c r="C8" s="11">
-        <f>B8*$B$3</f>
-      </c>
-      <c r="D8" s="12">
+      <c r="B8" s="11">
+        <v>4000</v>
+      </c>
+      <c r="C8" s="12">
         <v>1.5</v>
       </c>
-      <c r="E8" s="11">
-        <f>C8*D8</f>
+      <c r="D8" s="11">
+        <f>B8*C8</f>
+      </c>
+      <c r="E8" s="1">
+        <f>Pricing!E4</f>
       </c>
       <c r="F8" s="1">
-        <f>Pricing!E4</f>
+        <f>Pricing!C4</f>
       </c>
       <c r="G8" s="1">
-        <f>Pricing!C4</f>
-      </c>
-      <c r="H8" s="1">
-        <f>$B$4*F8+$B$5*G8</f>
+        <f>$B$3*E8+$B$4*F8</f>
+      </c>
+      <c r="H8" s="13">
+        <f>D8*G8</f>
       </c>
       <c r="I8" s="13">
-        <f>E8*H8</f>
-      </c>
-      <c r="J8" s="13">
-        <f>I8*12</f>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <f>H8*12</f>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="C9" s="11">
-        <f>B9*$B$3</f>
-      </c>
-      <c r="D9" s="12">
+      <c r="B9" s="11">
+        <v>500</v>
+      </c>
+      <c r="C9" s="12">
         <v>5</v>
       </c>
-      <c r="E9" s="11">
-        <f>C9*D9</f>
+      <c r="D9" s="11">
+        <f>B9*C9</f>
+      </c>
+      <c r="E9" s="1">
+        <f>Pricing!E5</f>
       </c>
       <c r="F9" s="1">
-        <f>Pricing!E5</f>
+        <f>Pricing!C5</f>
       </c>
       <c r="G9" s="1">
-        <f>Pricing!C5</f>
-      </c>
-      <c r="H9" s="1">
-        <f>$B$4*F9+$B$5*G9</f>
+        <f>$B$3*E9+$B$4*F9</f>
+      </c>
+      <c r="H9" s="13">
+        <f>D9*G9</f>
       </c>
       <c r="I9" s="13">
-        <f>E9*H9</f>
-      </c>
-      <c r="J9" s="13">
-        <f>I9*12</f>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+        <f>H9*12</f>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2">
-        <v>0.06</v>
-      </c>
-      <c r="C10" s="11">
-        <f>B10*$B$3</f>
-      </c>
-      <c r="D10" s="12">
+      <c r="B10" s="11">
+        <v>300</v>
+      </c>
+      <c r="C10" s="12">
         <v>13</v>
       </c>
-      <c r="E10" s="11">
-        <f>C10*D10</f>
+      <c r="D10" s="11">
+        <f>B10*C10</f>
+      </c>
+      <c r="E10" s="1">
+        <f>Pricing!E6</f>
       </c>
       <c r="F10" s="1">
-        <f>Pricing!E6</f>
+        <f>Pricing!C6</f>
       </c>
       <c r="G10" s="1">
-        <f>Pricing!C6</f>
-      </c>
-      <c r="H10" s="1">
-        <f>$B$4*F10+$B$5*G10</f>
+        <f>$B$3*E10+$B$4*F10</f>
+      </c>
+      <c r="H10" s="13">
+        <f>D10*G10</f>
       </c>
       <c r="I10" s="13">
-        <f>E10*H10</f>
-      </c>
-      <c r="J10" s="13">
-        <f>I10*12</f>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+        <f>H10*12</f>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="2">
-        <v>0.03</v>
-      </c>
-      <c r="C11" s="11">
-        <f>B11*$B$3</f>
-      </c>
-      <c r="D11" s="12">
+      <c r="B11" s="11">
+        <v>200</v>
+      </c>
+      <c r="C11" s="12">
         <v>30</v>
       </c>
-      <c r="E11" s="11">
-        <f>C11*D11</f>
+      <c r="D11" s="11">
+        <f>B11*C11</f>
+      </c>
+      <c r="E11" s="1">
+        <f>Pricing!E7</f>
       </c>
       <c r="F11" s="1">
-        <f>Pricing!E7</f>
+        <f>Pricing!C7</f>
       </c>
       <c r="G11" s="1">
-        <f>Pricing!C7</f>
-      </c>
-      <c r="H11" s="1">
-        <f>$B$4*F11+$B$5*G11</f>
+        <f>$B$3*E11+$B$4*F11</f>
+      </c>
+      <c r="H11" s="13">
+        <f>D11*G11</f>
       </c>
       <c r="I11" s="13">
-        <f>E11*H11</f>
-      </c>
-      <c r="J11" s="13">
-        <f>I11*12</f>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+        <f>H11*12</f>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="2">
-        <v>0.01</v>
-      </c>
-      <c r="C12" s="11">
-        <f>B12*$B$3</f>
-      </c>
-      <c r="D12" s="12">
+      <c r="B12" s="11">
+        <v>50</v>
+      </c>
+      <c r="C12" s="12">
         <v>75</v>
       </c>
-      <c r="E12" s="11">
-        <f>C12*D12</f>
-      </c>
-      <c r="F12" s="1">
-        <f>Pricing!E8</f>
-      </c>
-      <c r="G12" s="1">
-        <f>Pricing!C8</f>
-      </c>
-      <c r="H12" s="1">
-        <f>$B$4*F12+$B$5*G12</f>
+      <c r="D12" s="11">
+        <f>B12*C12</f>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" s="13">
+        <f>B12*$B$5</f>
       </c>
       <c r="I12" s="13">
-        <f>E12*H12</f>
-      </c>
-      <c r="J12" s="13">
-        <f>I12*12</f>
-      </c>
-    </row>
-    <row r="13" spans="1:10" s="17" customFormat="1" x14ac:dyDescent="0.25">
+        <f>H12*12</f>
+      </c>
+    </row>
+    <row r="13" spans="1:9" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B13" s="22">
         <f>SUM(B8:B12)</f>
       </c>
-      <c r="C13" s="23">
-        <f>SUM(C8:C12)</f>
-      </c>
-      <c r="D13" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="23">
-        <f>SUM(E8:E12)</f>
-      </c>
-      <c r="F13" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="G13" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="H13" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="I13" s="26">
+      <c r="C13" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="22">
+        <f>SUM(D8:D12)</f>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" s="25">
+        <f>SUM(H8:H12)</f>
+      </c>
+      <c r="I13" s="25">
         <f>SUM(I8:I12)</f>
       </c>
-      <c r="J13" s="26">
-        <f>SUM(J8:J12)</f>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>32</v>
+        <v>36</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="I15" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="J15" s="27">
-        <f>J13</f>
+        <v>35</v>
+      </c>
+      <c r="H15" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I15" s="26">
+        <f>I13</f>
       </c>
     </row>
   </sheetData>
@@ -1234,20 +1220,20 @@
   <sheetData>
     <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B3" s="1">
-        <f>'Revenue Model'!I13/'Revenue Model'!E13</f>
+        <f>'Revenue Model'!H13/'Revenue Model'!D13</f>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -1255,7 +1241,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2">
         <v>0.035</v>
@@ -1263,15 +1249,15 @@
     </row>
     <row r="6" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="28">
+        <v>41</v>
+      </c>
+      <c r="B6" s="27">
         <f>B3-B4-B3*B5</f>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B7" s="2">
         <f>B6/B3</f>
@@ -1279,31 +1265,31 @@
     </row>
     <row r="9" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B10" s="12">
-        <f>'Revenue Model'!E13/'Revenue Model'!C13</f>
+        <f>'Revenue Model'!D13/'Revenue Model'!B13</f>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B11" s="13">
-        <f>'Revenue Model'!I13/'Revenue Model'!C13</f>
+        <f>'Revenue Model'!H13/'Revenue Model'!B13</f>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B12" s="13">
         <f>B6*B10</f>
@@ -1311,15 +1297,15 @@
     </row>
     <row r="14" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B15" s="13">
         <v>150</v>
@@ -1327,7 +1313,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B16" s="2">
         <v>0.03</v>
@@ -1335,7 +1321,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B17" s="12">
         <f>1/B16</f>
@@ -1343,23 +1329,23 @@
     </row>
     <row r="18" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="29">
+        <v>51</v>
+      </c>
+      <c r="B18" s="28">
         <f>B12*B17</f>
       </c>
     </row>
     <row r="19" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="30" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" s="31">
+      <c r="A19" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="30">
         <f>B18/B15</f>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B20" s="12">
         <f>B15/B12</f>
@@ -1377,87 +1363,87 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="14" style="11" customWidth="1"/>
-    <col min="3" max="3" width="14" style="2" customWidth="1"/>
-    <col min="4" max="4" width="16" style="13" customWidth="1"/>
-    <col min="5" max="5" width="46" style="32" customWidth="1"/>
+    <col min="2" max="2" width="12" style="11" customWidth="1"/>
+    <col min="3" max="3" width="12" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14" style="13" customWidth="1"/>
+    <col min="5" max="5" width="48" style="31" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="5"/>
       <c r="D1" s="16"/>
-      <c r="E1" s="33"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="3" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="E3" s="34" t="s">
-        <v>56</v>
+        <v>58</v>
+      </c>
+      <c r="E3" s="33" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B4" s="11">
         <v>500</v>
       </c>
       <c r="C4" s="2">
-        <f>B4/5000</f>
+        <f>B4/5050</f>
       </c>
       <c r="D4" s="13">
-        <f>B4*('Revenue Model'!J13/'Revenue Model'!C13)</f>
-      </c>
-      <c r="E4" s="32" t="s">
-        <v>58</v>
+        <f>B4*('Revenue Model'!I13/'Revenue Model'!B13)</f>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B5" s="11">
         <v>2000</v>
       </c>
       <c r="C5" s="2">
-        <f>B5/5000</f>
+        <f>B5/5050</f>
       </c>
       <c r="D5" s="13">
-        <f>B5*('Revenue Model'!J13/'Revenue Model'!C13)</f>
-      </c>
-      <c r="E5" s="32" t="s">
-        <v>60</v>
+        <f>B5*('Revenue Model'!I13/'Revenue Model'!B13)</f>
+      </c>
+      <c r="E5" s="31" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B6" s="11">
-        <v>5000</v>
+        <v>5050</v>
       </c>
       <c r="C6" s="2">
-        <f>B6/5000</f>
+        <f>B6/5050</f>
       </c>
       <c r="D6" s="13">
-        <f>B6*('Revenue Model'!J13/'Revenue Model'!C13)</f>
-      </c>
-      <c r="E6" s="32" t="s">
-        <v>62</v>
+        <f>B6*('Revenue Model'!I13/'Revenue Model'!B13)</f>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1472,159 +1458,159 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="64" style="32" customWidth="1"/>
+    <col min="2" max="2" width="64" style="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
-        <v>63</v>
-      </c>
-      <c r="B1" s="36" t="s">
-        <v>32</v>
+    <row r="1" spans="1:2" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="35" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" s="32" t="s">
-        <v>65</v>
+        <v>67</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="32" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>32</v>
+        <v>69</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>67</v>
+        <v>71</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="32" t="s">
-        <v>69</v>
+        <v>8</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="32" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>32</v>
+        <v>10</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="32" t="s">
-        <v>72</v>
+        <v>14</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>73</v>
-      </c>
-      <c r="B10" s="32" t="s">
-        <v>74</v>
+        <v>16</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>75</v>
-      </c>
-      <c r="B11" s="32" t="s">
-        <v>76</v>
+        <v>77</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="32" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" s="36" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B14" s="32" t="s">
-        <v>79</v>
+        <v>80</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>80</v>
-      </c>
-      <c r="B15" s="32" t="s">
-        <v>81</v>
+        <v>82</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" s="32" t="s">
-        <v>83</v>
+        <v>84</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="32" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="35" t="s">
-        <v>84</v>
-      </c>
-      <c r="B18" s="36" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>85</v>
-      </c>
-      <c r="B19" s="32" t="s">
-        <v>86</v>
+        <v>88</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Condo Assistant: smooth pricing cliff with $500/mo cap; small-owner priority + PM-channel strategy (~$4.42M ARR)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_files/Condo_Assistant_SaaS_Model.xlsx
+++ b/project_files/Condo_Assistant_SaaS_Model.xlsx
@@ -15,9 +15,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="90">
-  <si>
-    <t>CONDO ASSISTANT — PRICING</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="89">
+  <si>
+    <t>CONDO ASSISTANT — PRICING (per unit / month)</t>
   </si>
   <si>
     <t>Band</t>
@@ -35,7 +35,7 @@
     <t>Bundle (Both)</t>
   </si>
   <si>
-    <t>Bundle Discount</t>
+    <t>Bundle Disc.</t>
   </si>
   <si>
     <t>Base</t>
@@ -53,72 +53,63 @@
     <t>Tier 2</t>
   </si>
   <si>
+    <t>10+ units</t>
+  </si>
+  <si>
+    <t>MONTHLY CAP: $500 per client (up to 100 units). 100+ units = custom quote.</t>
+  </si>
+  <si>
+    <t>The cap smooths the curve: a client's bill rises with units, then plateaus at $500 — it never drops as they add units. Big clients get a deep effective discount (75 units ≈ $6.67/unit).</t>
+  </si>
+  <si>
+    <t>REVENUE MODEL — at full penetration</t>
+  </si>
+  <si>
+    <t>Bundle Adoption %</t>
+  </si>
+  <si>
+    <t>Single-Product %</t>
+  </si>
+  <si>
+    <t>Monthly Cap / Client ($)</t>
+  </si>
+  <si>
+    <t># Clients</t>
+  </si>
+  <si>
+    <t>Avg Units</t>
+  </si>
+  <si>
+    <t>Total Units</t>
+  </si>
+  <si>
+    <t>Bundle $/u</t>
+  </si>
+  <si>
+    <t>Single $/u</t>
+  </si>
+  <si>
+    <t>Blended $/u</t>
+  </si>
+  <si>
+    <t>Bill/Client</t>
+  </si>
+  <si>
+    <t>Monthly Rev</t>
+  </si>
+  <si>
+    <t>Annual Rev</t>
+  </si>
+  <si>
     <t>10–19 units</t>
   </si>
   <si>
-    <t>Tier 3</t>
-  </si>
-  <si>
     <t>20–49 units</t>
   </si>
   <si>
-    <t>Enterprise</t>
-  </si>
-  <si>
     <t>50–100 units</t>
   </si>
   <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>FLAT $500/mo</t>
-  </si>
-  <si>
-    <t>Enterprise = clients with 50–100 units pay a flat $500/mo (≈$6.67/unit at 75 units). 100+ units = custom.</t>
-  </si>
-  <si>
-    <t>Single product = Condo Assistant OR Auto Email. Bundle = both. Bigger discount kicks in at 20+ units.</t>
-  </si>
-  <si>
-    <t>REVENUE MODEL — at full penetration</t>
-  </si>
-  <si>
-    <t>Bundle Adoption %</t>
-  </si>
-  <si>
-    <t>Single-Product %</t>
-  </si>
-  <si>
-    <t>Enterprise Flat Rate ($/mo)</t>
-  </si>
-  <si>
-    <t># Clients</t>
-  </si>
-  <si>
-    <t>Avg Units</t>
-  </si>
-  <si>
-    <t>Total Units</t>
-  </si>
-  <si>
-    <t>Bundle $/u</t>
-  </si>
-  <si>
-    <t>Single $/u</t>
-  </si>
-  <si>
-    <t>Blended $/u</t>
-  </si>
-  <si>
-    <t>Monthly Rev</t>
-  </si>
-  <si>
-    <t>Annual Rev</t>
-  </si>
-  <si>
-    <t>flat</t>
-  </si>
-  <si>
     <t>TOTAL</t>
   </si>
   <si>
@@ -200,13 +191,13 @@
     <t>Year 1</t>
   </si>
   <si>
-    <t>Pilot &amp; early adopters — WPM referrals, CO STR groups, host DMs (near-zero CAC)</t>
+    <t>Pilot — small owners via WPM referrals + CO STR groups (near-zero CAC)</t>
   </si>
   <si>
     <t>Year 2</t>
   </si>
   <si>
-    <t>Scale — PM/software partners + Escapia/Guesty affiliates (Option C)</t>
+    <t>Land large PM companies (Option C) — they refer &amp; credential the small owners</t>
   </si>
   <si>
     <t>Year 3</t>
@@ -218,16 +209,43 @@
     <t>PRICING</t>
   </si>
   <si>
-    <t>Per-unit bands</t>
-  </si>
-  <si>
-    <t>1–2 $25 · 3–9 $22 · 10–19 $20 · 20–49 $14 (bundle). Single product ~$6 less. Bigger discount at 20+.</t>
-  </si>
-  <si>
-    <t>Enterprise (50–100 units)</t>
-  </si>
-  <si>
-    <t>FLAT $500/mo per client (≈$6.67/unit at 75 units). 100+ units = custom quote.</t>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>Condo Assistant $15/unit · Auto Email $15/unit · Bundle (both) $25/unit (base)</t>
+  </si>
+  <si>
+    <t>Volume tiers (bundle)</t>
+  </si>
+  <si>
+    <t>1–2 units $25 · 3–9 $22 · 10+ $20 per unit</t>
+  </si>
+  <si>
+    <t>Monthly cap</t>
+  </si>
+  <si>
+    <t>$500/client up to 100 units. This smooths the cliff — the bill plateaus at $500, never drops. 100+ = custom.</t>
+  </si>
+  <si>
+    <t>Effective enterprise discount</t>
+  </si>
+  <si>
+    <t>A 75-unit client at the $500 cap pays ≈$6.67/unit (73% off) — deep discount to land large managers.</t>
+  </si>
+  <si>
+    <t>STRATEGY</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Under-5-unit owners — most profitable per unit, biggest segment (4,000 of 5,050 clients).</t>
+  </si>
+  <si>
+    <t>Large managers = channel</t>
+  </si>
+  <si>
+    <t>Big PM companies (20–100 units) are priced aggressively (capped) because their adoption + referrals make the small, profitable owners easier &amp; cheaper to land.</t>
   </si>
   <si>
     <t>CLIENT DISTRIBUTION (your numbers)</t>
@@ -236,22 +254,13 @@
     <t>4,000 clients</t>
   </si>
   <si>
-    <t>500 clients</t>
-  </si>
-  <si>
-    <t>300 clients</t>
-  </si>
-  <si>
-    <t>200 clients</t>
-  </si>
-  <si>
-    <t>50 clients (seeded — the "rest"; adjust as needed)</t>
+    <t>500 · 10–19: 300 · 20–49: 200 · 50–100: 50 (seeded "rest") = 5,050 total</t>
   </si>
   <si>
     <t>Avg units/client</t>
   </si>
   <si>
-    <t>Illustrative per band (1.5 / 5 / 13 / 30 / 75) — refine with real data</t>
+    <t>Illustrative (1.5 / 5 / 13 / 30 / 75) — refine with real data</t>
   </si>
   <si>
     <t>UNIT ECONOMICS</t>
@@ -260,31 +269,19 @@
     <t>COGS/unit/mo</t>
   </si>
   <si>
-    <t>$3 placeholder — Claude API + hosting + Resend email</t>
-  </si>
-  <si>
-    <t>Stripe</t>
-  </si>
-  <si>
-    <t>~3.5% blended (2.9% + $0.30/txn)</t>
-  </si>
-  <si>
-    <t>CAC / churn</t>
-  </si>
-  <si>
-    <t>$150 CAC, 3% monthly churn — illustrative</t>
-  </si>
-  <si>
-    <t>NOTE — pricing cliff</t>
-  </si>
-  <si>
-    <t>A 49-unit client (per-unit) can pay more than a 50-unit client (flat $500). Intentional "graduate to enterprise" discount, but watch the boundary.</t>
+    <t>$3 placeholder (Claude API + hosting + Resend)</t>
+  </si>
+  <si>
+    <t>Stripe / CAC / churn</t>
+  </si>
+  <si>
+    <t>~3.5% / $150 / 3% monthly — illustrative</t>
   </si>
   <si>
     <t>All numbers illustrative</t>
   </si>
   <si>
-    <t>Planning model to show Alex. Replace estimates with real data as it comes in.</t>
+    <t>Planning model for Alex — this is a first-pass guess. Replace estimates with real data as it comes in.</t>
   </si>
 </sst>
 </file>
@@ -297,7 +294,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -312,6 +309,10 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1F3864"/>
     </font>
     <font>
       <color rgb="FF777777"/>
@@ -359,7 +360,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -371,26 +372,27 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -400,8 +402,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -743,13 +745,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="1" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
     <col min="4" max="4" width="16" style="1" customWidth="1"/>
-    <col min="5" max="5" width="20" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18" style="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="2" customWidth="1"/>
   </cols>
   <sheetData>
@@ -842,54 +844,14 @@
         <f>1-E6/$E$4</f>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="8" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="9" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
         <v>14</v>
-      </c>
-      <c r="C7" s="1">
-        <v>9</v>
-      </c>
-      <c r="D7" s="1">
-        <v>9</v>
-      </c>
-      <c r="E7" s="1">
-        <v>14</v>
-      </c>
-      <c r="F7" s="2">
-        <f>1-E7/$E$4</f>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="2">
-        <f>1-(500/75)/E4</f>
-      </c>
-    </row>
-    <row r="10" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -900,117 +862,124 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="12" style="11" customWidth="1"/>
-    <col min="3" max="3" width="14" style="12" customWidth="1"/>
-    <col min="4" max="4" width="12" style="11" customWidth="1"/>
-    <col min="5" max="5" width="14" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14" style="1" customWidth="1"/>
-    <col min="8" max="9" width="16" style="13" customWidth="1"/>
+    <col min="2" max="2" width="11" style="12" customWidth="1"/>
+    <col min="3" max="3" width="11" style="13" customWidth="1"/>
+    <col min="4" max="4" width="12" style="12" customWidth="1"/>
+    <col min="5" max="6" width="11" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13" style="14" customWidth="1"/>
+    <col min="9" max="10" width="15" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="14"/>
+        <v>15</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="11">
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="12">
         <v>0.65</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="11"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="12"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="11">
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="12">
         <f>1-B3</f>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="11"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="12"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="11">
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="12">
         <v>500</v>
       </c>
-      <c r="C5" s="12"/>
-      <c r="D5" s="11"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="12"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-    </row>
-    <row r="7" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+    </row>
+    <row r="7" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="I7" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="J7" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="I7" s="20" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="12">
         <v>4000</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="13">
         <v>1.5</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="12">
         <f>B8*C8</f>
       </c>
       <c r="E8" s="1">
@@ -1022,24 +991,27 @@
       <c r="G8" s="1">
         <f>$B$3*E8+$B$4*F8</f>
       </c>
-      <c r="H8" s="13">
-        <f>D8*G8</f>
-      </c>
-      <c r="I8" s="13">
-        <f>H8*12</f>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H8" s="14">
+        <f>MIN(C8*G8,$B$5)</f>
+      </c>
+      <c r="I8" s="14">
+        <f>B8*H8</f>
+      </c>
+      <c r="J8" s="14">
+        <f>I8*12</f>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="12">
         <v>500</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="13">
         <v>5</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="12">
         <f>B9*C9</f>
       </c>
       <c r="E9" s="1">
@@ -1051,24 +1023,27 @@
       <c r="G9" s="1">
         <f>$B$3*E9+$B$4*F9</f>
       </c>
-      <c r="H9" s="13">
-        <f>D9*G9</f>
-      </c>
-      <c r="I9" s="13">
-        <f>H9*12</f>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H9" s="14">
+        <f>MIN(C9*G9,$B$5)</f>
+      </c>
+      <c r="I9" s="14">
+        <f>B9*H9</f>
+      </c>
+      <c r="J9" s="14">
+        <f>I9*12</f>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="11">
+        <v>28</v>
+      </c>
+      <c r="B10" s="12">
         <v>300</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="13">
         <v>13</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="12">
         <f>B10*C10</f>
       </c>
       <c r="E10" s="1">
@@ -1080,127 +1055,142 @@
       <c r="G10" s="1">
         <f>$B$3*E10+$B$4*F10</f>
       </c>
-      <c r="H10" s="13">
-        <f>D10*G10</f>
-      </c>
-      <c r="I10" s="13">
-        <f>H10*12</f>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H10" s="14">
+        <f>MIN(C10*G10,$B$5)</f>
+      </c>
+      <c r="I10" s="14">
+        <f>B10*H10</f>
+      </c>
+      <c r="J10" s="14">
+        <f>I10*12</f>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="11">
+        <v>29</v>
+      </c>
+      <c r="B11" s="12">
         <v>200</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="13">
         <v>30</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="12">
         <f>B11*C11</f>
       </c>
       <c r="E11" s="1">
-        <f>Pricing!E7</f>
+        <f>Pricing!E6</f>
       </c>
       <c r="F11" s="1">
-        <f>Pricing!C7</f>
+        <f>Pricing!C6</f>
       </c>
       <c r="G11" s="1">
         <f>$B$3*E11+$B$4*F11</f>
       </c>
-      <c r="H11" s="13">
-        <f>D11*G11</f>
-      </c>
-      <c r="I11" s="13">
-        <f>H11*12</f>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H11" s="14">
+        <f>MIN(C11*G11,$B$5)</f>
+      </c>
+      <c r="I11" s="14">
+        <f>B11*H11</f>
+      </c>
+      <c r="J11" s="14">
+        <f>I11*12</f>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="11">
+        <v>30</v>
+      </c>
+      <c r="B12" s="12">
         <v>50</v>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="13">
         <v>75</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="12">
         <f>B12*C12</f>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="1">
+        <f>Pricing!E6</f>
+      </c>
+      <c r="F12" s="1">
+        <f>Pricing!C6</f>
+      </c>
+      <c r="G12" s="1">
+        <f>$B$3*E12+$B$4*F12</f>
+      </c>
+      <c r="H12" s="14">
+        <f>MIN(C12*G12,$B$5)</f>
+      </c>
+      <c r="I12" s="14">
+        <f>B12*H12</f>
+      </c>
+      <c r="J12" s="14">
+        <f>I12*12</f>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="23">
+        <f>SUM(B8:B12)</f>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="23">
+        <f>SUM(D8:D12)</f>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="H13" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="26">
+        <f>SUM(I8:I12)</f>
+      </c>
+      <c r="J13" s="26">
+        <f>SUM(J8:J12)</f>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H12" s="13">
-        <f>B12*$B$5</f>
-      </c>
-      <c r="I12" s="13">
-        <f>H12*12</f>
-      </c>
-    </row>
-    <row r="13" spans="1:9" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="22">
-        <f>SUM(B8:B12)</f>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="22">
-        <f>SUM(D8:D12)</f>
-      </c>
-      <c r="E13" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="G13" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="H13" s="25">
-        <f>SUM(H8:H12)</f>
-      </c>
-      <c r="I13" s="25">
-        <f>SUM(I8:I12)</f>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>35</v>
+      <c r="B15" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>32</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H15" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="I15" s="26">
-        <f>I13</f>
+        <v>32</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="J15" s="27">
+        <f>J13</f>
       </c>
     </row>
   </sheetData>
@@ -1220,20 +1210,20 @@
   <sheetData>
     <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B3" s="1">
-        <f>'Revenue Model'!H13/'Revenue Model'!D13</f>
+        <f>'Revenue Model'!I13/'Revenue Model'!D13</f>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -1241,79 +1231,79 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B5" s="2">
         <v>0.035</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="27">
+    <row r="6" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="28">
         <f>B3-B4-B3*B5</f>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B7" s="2">
         <f>B6/B3</f>
       </c>
     </row>
-    <row r="9" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>35</v>
+    <row r="9" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="12">
+        <v>41</v>
+      </c>
+      <c r="B10" s="13">
         <f>'Revenue Model'!D13/'Revenue Model'!B13</f>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="13">
-        <f>'Revenue Model'!H13/'Revenue Model'!B13</f>
+        <v>42</v>
+      </c>
+      <c r="B11" s="14">
+        <f>'Revenue Model'!I13/'Revenue Model'!B13</f>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="13">
+        <v>43</v>
+      </c>
+      <c r="B12" s="14">
         <f>B6*B10</f>
       </c>
     </row>
-    <row r="14" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>35</v>
+    <row r="14" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="13">
+        <v>45</v>
+      </c>
+      <c r="B15" s="14">
         <v>150</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B16" s="2">
         <v>0.03</v>
@@ -1321,33 +1311,33 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" s="12">
+        <v>47</v>
+      </c>
+      <c r="B17" s="13">
         <f>1/B16</f>
       </c>
     </row>
-    <row r="18" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" s="28">
+    <row r="18" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="29">
         <f>B12*B17</f>
       </c>
     </row>
-    <row r="19" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="B19" s="30">
+    <row r="19" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="31">
         <f>B18/B15</f>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="12">
+        <v>50</v>
+      </c>
+      <c r="B20" s="13">
         <f>B15/B12</f>
       </c>
     </row>
@@ -1363,87 +1353,87 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="12" style="11" customWidth="1"/>
+    <col min="2" max="2" width="12" style="12" customWidth="1"/>
     <col min="3" max="3" width="12" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14" style="13" customWidth="1"/>
-    <col min="5" max="5" width="48" style="31" customWidth="1"/>
+    <col min="4" max="4" width="14" style="14" customWidth="1"/>
+    <col min="5" max="5" width="50" style="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B1" s="14"/>
+        <v>51</v>
+      </c>
+      <c r="B1" s="15"/>
       <c r="C1" s="5"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="32"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="3" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="E3" s="34" t="s">
         <v>56</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="E3" s="33" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="11">
+        <v>57</v>
+      </c>
+      <c r="B4" s="12">
         <v>500</v>
       </c>
       <c r="C4" s="2">
         <f>B4/5050</f>
       </c>
-      <c r="D4" s="13">
-        <f>B4*('Revenue Model'!I13/'Revenue Model'!B13)</f>
-      </c>
-      <c r="E4" s="31" t="s">
-        <v>61</v>
+      <c r="D4" s="14">
+        <f>B4*('Revenue Model'!J13/'Revenue Model'!B13)</f>
+      </c>
+      <c r="E4" s="32" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="11">
+        <v>59</v>
+      </c>
+      <c r="B5" s="12">
         <v>2000</v>
       </c>
       <c r="C5" s="2">
         <f>B5/5050</f>
       </c>
-      <c r="D5" s="13">
-        <f>B5*('Revenue Model'!I13/'Revenue Model'!B13)</f>
-      </c>
-      <c r="E5" s="31" t="s">
-        <v>63</v>
+      <c r="D5" s="14">
+        <f>B5*('Revenue Model'!J13/'Revenue Model'!B13)</f>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="11">
+        <v>61</v>
+      </c>
+      <c r="B6" s="12">
         <v>5050</v>
       </c>
       <c r="C6" s="2">
         <f>B6/5050</f>
       </c>
-      <c r="D6" s="13">
-        <f>B6*('Revenue Model'!I13/'Revenue Model'!B13)</f>
-      </c>
-      <c r="E6" s="31" t="s">
-        <v>65</v>
+      <c r="D6" s="14">
+        <f>B6*('Revenue Model'!J13/'Revenue Model'!B13)</f>
+      </c>
+      <c r="E6" s="32" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1454,163 +1444,171 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="64" style="31" customWidth="1"/>
+    <col min="2" max="2" width="64" style="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
-        <v>66</v>
-      </c>
-      <c r="B1" s="35" t="s">
-        <v>35</v>
+    <row r="1" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="36" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>68</v>
+        <v>64</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B3" s="31" t="s">
-        <v>70</v>
+        <v>66</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="31" t="s">
-        <v>35</v>
+        <v>68</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="32" t="s">
         <v>71</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="35" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>73</v>
+      <c r="B7" s="36" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="31" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="32" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="31" t="s">
         <v>75</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="31" t="s">
-        <v>76</v>
+        <v>32</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>77</v>
       </c>
-      <c r="B11" s="31" t="s">
-        <v>78</v>
+      <c r="B11" s="32" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="31" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="32" t="s">
         <v>79</v>
-      </c>
-      <c r="B13" s="35" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="32" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="32" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="31" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>84</v>
-      </c>
-      <c r="B16" s="31" t="s">
-        <v>85</v>
+      <c r="B16" s="36" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B17" s="31" t="s">
-        <v>35</v>
+        <v>83</v>
+      </c>
+      <c r="B17" s="32" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="32" t="s">
         <v>86</v>
-      </c>
-      <c r="B18" s="31" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="32" t="s">
         <v>88</v>
-      </c>
-      <c r="B19" s="31" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Condo Assistant model: add COGS breakdown tab (AI chat+email, hosting, email, embeddings = $3/unit)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_files/Condo_Assistant_SaaS_Model.xlsx
+++ b/project_files/Condo_Assistant_SaaS_Model.xlsx
@@ -9,13 +9,14 @@
     <sheet sheetId="3" name="Unit Economics" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Rollout Ramp" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Assumptions &amp; Notes" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="COGS Breakdown" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="107">
   <si>
     <t>CONDO ASSISTANT — PRICING (per unit / month)</t>
   </si>
@@ -125,7 +126,7 @@
     <t>Avg Revenue / Unit / Month</t>
   </si>
   <si>
-    <t>COGS / Unit / Month (AI + hosting + email)</t>
+    <t>COGS / Unit / Month (from COGS Breakdown)</t>
   </si>
   <si>
     <t>Stripe Fee (% of revenue)</t>
@@ -282,6 +283,60 @@
   </si>
   <si>
     <t>Planning model for Alex — this is a first-pass guess. Replace estimates with real data as it comes in.</t>
+  </si>
+  <si>
+    <t>COGS BREAKDOWN (per unit / month)</t>
+  </si>
+  <si>
+    <t>Cost Component</t>
+  </si>
+  <si>
+    <t>$ / Unit / Mo</t>
+  </si>
+  <si>
+    <t>Basis</t>
+  </si>
+  <si>
+    <t>Guest chat AI (Claude Haiku 4.5)</t>
+  </si>
+  <si>
+    <t>~90 questions/mo (6 res × 15 Q), ~4.2K tokens each @ $1/$5 per M</t>
+  </si>
+  <si>
+    <t>Auto Email AI (Claude Haiku 4.5)</t>
+  </si>
+  <si>
+    <t>~100 AI replies/mo (200-email thread), ~5.35K tokens each</t>
+  </si>
+  <si>
+    <t>Hosting (Vercel + Supabase, amortized)</t>
+  </si>
+  <si>
+    <t>App hosting + Postgres/pgvector, spread per unit</t>
+  </si>
+  <si>
+    <t>Email delivery (Resend)</t>
+  </si>
+  <si>
+    <t>Transactional + auto-reply sends</t>
+  </si>
+  <si>
+    <t>Embeddings (OpenAI, RAG)</t>
+  </si>
+  <si>
+    <t>Query embeddings per message (near-zero)</t>
+  </si>
+  <si>
+    <t>Buffer / overage</t>
+  </si>
+  <si>
+    <t>Headroom for spikes, Sonnet upgrade, growth</t>
+  </si>
+  <si>
+    <t>TOTAL COGS / Unit / Month</t>
+  </si>
+  <si>
+    <t>Model: Claude Haiku 4.5 ($1/M in · $5/M out). Sonnet 5 upgrade ≈ 3× the AI lines. Estimates — calibrate with real prompt sizes via count_tokens.</t>
   </si>
 </sst>
 </file>
@@ -360,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -405,6 +460,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1226,7 +1284,7 @@
         <v>36</v>
       </c>
       <c r="B4" s="1">
-        <v>3</v>
+        <f>'COGS Breakdown'!B10</f>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1615,4 +1673,115 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="52" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0.45</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.68</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="25">
+        <f>SUM(B3:B8)</f>
+      </c>
+    </row>
+    <row r="12" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="37" t="s">
+        <v>106</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Condo Assistant model: add $ at Scale tab (revenue/COGS/gross profit at 1K/5K/10K/22K units)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_files/Condo_Assistant_SaaS_Model.xlsx
+++ b/project_files/Condo_Assistant_SaaS_Model.xlsx
@@ -10,13 +10,14 @@
     <sheet sheetId="4" name="Rollout Ramp" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Assumptions &amp; Notes" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="COGS Breakdown" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="$ at Scale" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="123">
   <si>
     <t>CONDO ASSISTANT — PRICING (per unit / month)</t>
   </si>
@@ -337,6 +338,54 @@
   </si>
   <si>
     <t>Model: Claude Haiku 4.5 ($1/M in · $5/M out). Sonnet 5 upgrade ≈ 3× the AI lines. Estimates — calibrate with real prompt sizes via count_tokens.</t>
+  </si>
+  <si>
+    <t>$ AT SCALE — absolute dollars by fleet size</t>
+  </si>
+  <si>
+    <t>Per-Unit Drivers (live from model)</t>
+  </si>
+  <si>
+    <t>Avg Revenue / Unit / Mo</t>
+  </si>
+  <si>
+    <t>COGS / Unit / Mo</t>
+  </si>
+  <si>
+    <t>Stripe % of Revenue</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>1,000 units</t>
+  </si>
+  <si>
+    <t>5,000 units</t>
+  </si>
+  <si>
+    <t>10,000 units</t>
+  </si>
+  <si>
+    <t>Full (22,150)</t>
+  </si>
+  <si>
+    <t>Monthly Revenue</t>
+  </si>
+  <si>
+    <t>Monthly COGS</t>
+  </si>
+  <si>
+    <t>Monthly Stripe Fees</t>
+  </si>
+  <si>
+    <t>Monthly Gross Profit</t>
+  </si>
+  <si>
+    <t>Annual Gross Profit</t>
+  </si>
+  <si>
+    <t>Assumes the same blended per-unit economics as the full model (~$16.63 avg rev/unit — reflects the $500 enterprise caps). Early-stage fleets skew to small owners with higher avg $/unit, so these are conservative.</t>
   </si>
 </sst>
 </file>
@@ -415,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -464,6 +513,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1784,4 +1834,198 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" s="1">
+        <f>'Revenue Model'!I13/'Revenue Model'!D13</f>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="1">
+        <f>'COGS Breakdown'!B10</f>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="12">
+        <v>1000</v>
+      </c>
+      <c r="C9" s="12">
+        <v>5000</v>
+      </c>
+      <c r="D9" s="12">
+        <v>10000</v>
+      </c>
+      <c r="E9" s="12">
+        <v>22150</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B10" s="14">
+        <f>B9*$B$4</f>
+      </c>
+      <c r="C10" s="14">
+        <f>C9*$B$4</f>
+      </c>
+      <c r="D10" s="14">
+        <f>D9*$B$4</f>
+      </c>
+      <c r="E10" s="14">
+        <f>E9*$B$4</f>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B11" s="14">
+        <f>B9*$B$5</f>
+      </c>
+      <c r="C11" s="14">
+        <f>C9*$B$5</f>
+      </c>
+      <c r="D11" s="14">
+        <f>D9*$B$5</f>
+      </c>
+      <c r="E11" s="14">
+        <f>E9*$B$5</f>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" s="14">
+        <f>B10*$B$6</f>
+      </c>
+      <c r="C12" s="14">
+        <f>C10*$B$6</f>
+      </c>
+      <c r="D12" s="14">
+        <f>D10*$B$6</f>
+      </c>
+      <c r="E12" s="14">
+        <f>E10*$B$6</f>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="26">
+        <f>B10-B11-B12</f>
+      </c>
+      <c r="C13" s="26">
+        <f>C10-C11-C12</f>
+      </c>
+      <c r="D13" s="26">
+        <f>D10-D11-D12</f>
+      </c>
+      <c r="E13" s="26">
+        <f>E10-E11-E12</f>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="30" t="s">
+        <v>121</v>
+      </c>
+      <c r="B14" s="38">
+        <f>B13*12</f>
+      </c>
+      <c r="C14" s="38">
+        <f>C13*12</f>
+      </c>
+      <c r="D14" s="38">
+        <f>D13*12</f>
+      </c>
+      <c r="E14" s="38">
+        <f>E13*12</f>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="2">
+        <f>B13/B10</f>
+      </c>
+      <c r="C15" s="2">
+        <f>C13/C10</f>
+      </c>
+      <c r="D15" s="2">
+        <f>D13/D10</f>
+      </c>
+      <c r="E15" s="2">
+        <f>E13/E10</f>
+      </c>
+    </row>
+    <row r="17" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="37" t="s">
+        <v>122</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>